<commit_message>
Update hydraulic classes and salinity analysis assets
</commit_message>
<xml_diff>
--- a/literature_data/Photsynthesis and Stomatal Conductance Reduction Data.xlsx
+++ b/literature_data/Photsynthesis and Stomatal Conductance Reduction Data.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://geosyntec-my.sharepoint.com/personal/josh_gottlieb_geosyntec_com/Documents/Documents/SourceCode/Photo3-Plant-Salinity-Traits/literature_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="8_{A221A28E-6D81-423C-BE1B-F549E3B52D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C75FAA5-7510-4515-B581-5A902F91CCEE}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="8_{A221A28E-6D81-423C-BE1B-F549E3B52D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B37F8141-E142-4D72-8545-03DA3456C460}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-22416" yWindow="624" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{C0AAE20D-2553-4379-8EED-88D25BB078BE}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="2" xr2:uid="{C0AAE20D-2553-4379-8EED-88D25BB078BE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sanchez-Ledema Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Campos-Villareal Data" sheetId="3" r:id="rId2"/>
-    <sheet name="Photosynthetic Rate Reduct Plot" sheetId="2" r:id="rId3"/>
-    <sheet name="Photosynthetic Pct Reduct" sheetId="5" r:id="rId4"/>
-    <sheet name="Stomatal Conductance Reduc Plot" sheetId="4" r:id="rId5"/>
+    <sheet name="Sanchez-Ledesma Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Cao et al Data" sheetId="6" r:id="rId2"/>
+    <sheet name="Campos-Villareal Data" sheetId="3" r:id="rId3"/>
+    <sheet name="Photosynthetic Rate Reduct Plot" sheetId="2" r:id="rId4"/>
+    <sheet name="Photosynthetic Pct Reduct" sheetId="5" r:id="rId5"/>
+    <sheet name="Stomatal Conductance Reduc Plot" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -331,7 +332,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>'Sanchez-Ledema Data'!$C$2:$C$6</c:f>
+                <c:f>'Sanchez-Ledesma Data'!$C$2:$C$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="5"/>
@@ -355,7 +356,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>'Sanchez-Ledema Data'!$C$2:$C$6</c:f>
+                <c:f>'Sanchez-Ledesma Data'!$C$2:$C$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="5"/>
@@ -393,7 +394,7 @@
           </c:errBars>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$A$2:$A$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -417,7 +418,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$B$2:$B$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1242,7 +1243,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>'Sanchez-Ledema Data'!$C$2:$C$6</c:f>
+                <c:f>'Sanchez-Ledesma Data'!$C$2:$C$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="5"/>
@@ -1266,7 +1267,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>'Sanchez-Ledema Data'!$C$2:$C$6</c:f>
+                <c:f>'Sanchez-Ledesma Data'!$C$2:$C$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="5"/>
@@ -1304,7 +1305,7 @@
           </c:errBars>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$A$2:$A$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1328,7 +1329,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$E$2:$E$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$E$2:$E$6</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2225,7 +2226,7 @@
           </c:errBars>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$A$2:$A$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2249,7 +2250,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sanchez-Ledema Data'!$F$2:$F$6</c:f>
+              <c:f>'Sanchez-Ledesma Data'!$F$2:$F$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -5325,6 +5326,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4A21305-A9F1-4CBD-97D5-E3BBC3914A4F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD3CF77E-8971-4EF4-9E6E-8FC73109F299}">
   <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5448,7 +5458,7 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:O6" si="0">1-H3</f>
+        <f t="shared" ref="L3:N6" si="0">1-H3</f>
         <v>0</v>
       </c>
       <c r="M3">
@@ -5517,7 +5527,7 @@
         <v>0.18154761904761896</v>
       </c>
       <c r="O4" s="6">
-        <f t="shared" ref="O4:O6" si="3">AVERAGE(K4:N4)</f>
+        <f t="shared" ref="O4:O5" si="3">AVERAGE(K4:N4)</f>
         <v>0.23659766859836692</v>
       </c>
     </row>

</xml_diff>